<commit_message>
chore: fechamento do dia
</commit_message>
<xml_diff>
--- a/outputs_cepal/main_statistics_EN.xlsx
+++ b/outputs_cepal/main_statistics_EN.xlsx
@@ -1,164 +1,154 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/82aed305ce3fc73d/Documentos/UnB/Projetos/50_anos_cepal/cepal50anos/outputs_cepal/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_81C17C008CE9A86E58902791E24D42B133B8A413" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAA16489-9632-400F-B63E-481E54D43AD0}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
-    <t>Variable</t>
-  </si>
-  <si>
-    <t>Sigla</t>
-  </si>
-  <si>
-    <t>WoS</t>
-  </si>
-  <si>
-    <t>Scopus</t>
-  </si>
-  <si>
-    <t>Merged</t>
-  </si>
-  <si>
-    <t>Period (start year)</t>
-  </si>
-  <si>
-    <t>Years_start</t>
-  </si>
-  <si>
-    <t>Period (end year)</t>
-  </si>
-  <si>
-    <t>Years_end</t>
-  </si>
-  <si>
-    <t>Total Documents</t>
-  </si>
-  <si>
-    <t>GTP</t>
-  </si>
-  <si>
-    <t>Total Authors</t>
-  </si>
-  <si>
-    <t>GTA</t>
-  </si>
-  <si>
-    <t>Total Citations</t>
-  </si>
-  <si>
-    <t>GTC</t>
-  </si>
-  <si>
-    <t>Single-authored Documents</t>
-  </si>
-  <si>
-    <t>TP1</t>
-  </si>
-  <si>
-    <t>Multi-authored Documents</t>
-  </si>
-  <si>
-    <t>TPm</t>
-  </si>
-  <si>
-    <t>Authors of Single-authored Documents</t>
-  </si>
-  <si>
-    <t>TA1</t>
-  </si>
-  <si>
-    <t>Authors of Multi-authored Documents</t>
-  </si>
-  <si>
-    <t>TAm</t>
-  </si>
-  <si>
-    <t>Author Appearances</t>
-  </si>
-  <si>
-    <t>TAapp</t>
-  </si>
-  <si>
-    <t>Documents per Year</t>
-  </si>
-  <si>
-    <t>ADy</t>
-  </si>
-  <si>
-    <t>Documents per Author</t>
-  </si>
-  <si>
-    <t>ADa</t>
-  </si>
-  <si>
-    <t>Authors per Document</t>
-  </si>
-  <si>
-    <t>AAd</t>
-  </si>
-  <si>
-    <t>Co-authors per Document</t>
-  </si>
-  <si>
-    <t>ACAd</t>
-  </si>
-  <si>
-    <t>Collaboration Index</t>
-  </si>
-  <si>
-    <t>CI</t>
-  </si>
-  <si>
-    <t>Citations per Document</t>
-  </si>
-  <si>
-    <t>ACd</t>
-  </si>
-  <si>
-    <t>Collection h-index</t>
-  </si>
-  <si>
-    <t>h_collection</t>
-  </si>
-  <si>
-    <t>Authors' Keywords</t>
-  </si>
-  <si>
-    <t>GTKde</t>
-  </si>
-  <si>
-    <t>Keywords Plus</t>
-  </si>
-  <si>
-    <t>GTKid</t>
+    <t xml:space="preserve">Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sigla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WoS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scopus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period (start year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Years_start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period (end year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Years_end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Documents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GTP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Authors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Citations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GTC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single-authored Documents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TP1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multi-authored Documents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors of Single-authored Documents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TA1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors of Multi-authored Documents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Author Appearances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAapp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documents per Year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documents per Author</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors per Document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-authors per Document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACAd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collaboration Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citations per Document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collection h-index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h_collection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors' Keywords</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GTKde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keywords Plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GTKid</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="0.0"/>
-  </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -187,35 +177,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:E20" totalsRowShown="0">
-  <autoFilter ref="A1:E20" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:E20" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E20"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Variable"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Sigla"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="WoS"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Scopus"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Merged"/>
+    <tableColumn id="1" name="Variable"/>
+    <tableColumn id="2" name="Sigla"/>
+    <tableColumn id="3" name="WoS"/>
+    <tableColumn id="4" name="Scopus"/>
+    <tableColumn id="5" name="Merged"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -499,11 +479,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -520,334 +500,334 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>2007</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>1977</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>1977</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>2024</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>2025</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>2025</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>564</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>689</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>1168</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" t="s">
         <v>11</v>
       </c>
       <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>950</v>
       </c>
-      <c r="D5">
-        <v>987</v>
-      </c>
-      <c r="E5">
+      <c r="D5" t="n">
+        <v>985</v>
+      </c>
+      <c r="E5" t="n">
         <v>1833</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" t="s">
         <v>13</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>1405</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>2462</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>3329</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7">
       <c r="A7" t="s">
         <v>15</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>184</v>
       </c>
-      <c r="D7">
-        <v>267</v>
-      </c>
-      <c r="E7">
+      <c r="D7" t="n">
+        <v>264</v>
+      </c>
+      <c r="E7" t="n">
         <v>405</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8">
       <c r="A8" t="s">
         <v>17</v>
       </c>
       <c r="B8" t="s">
         <v>18</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>380</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>422</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>760</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9">
       <c r="A9" t="s">
         <v>19</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>153</v>
       </c>
-      <c r="D9">
-        <v>207</v>
-      </c>
-      <c r="E9">
+      <c r="D9" t="n">
+        <v>205</v>
+      </c>
+      <c r="E9" t="n">
         <v>329</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10">
       <c r="A10" t="s">
         <v>21</v>
       </c>
       <c r="B10" t="s">
         <v>22</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>829</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>823</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>1578</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11">
       <c r="A11" t="s">
         <v>23</v>
       </c>
       <c r="B11" t="s">
         <v>24</v>
       </c>
-      <c r="C11">
+      <c r="C11" t="n">
         <v>1172</v>
       </c>
-      <c r="D11">
-        <v>1356</v>
-      </c>
-      <c r="E11">
+      <c r="D11" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E11" t="n">
         <v>2378</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12">
       <c r="A12" t="s">
         <v>25</v>
       </c>
       <c r="B12" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" t="n">
         <v>31.3333333333333</v>
       </c>
-      <c r="D12" s="1">
-        <v>22.966666666666701</v>
-      </c>
-      <c r="E12" s="1">
-        <v>38.933333333333302</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D12" t="n">
+        <v>22.9666666666667</v>
+      </c>
+      <c r="E12" t="n">
+        <v>38.9333333333333</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" t="s">
         <v>27</v>
       </c>
       <c r="B13" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="1">
-        <v>0.59368421052631604</v>
-      </c>
-      <c r="D13" s="1">
-        <v>0.698074974670719</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0.63720676486633898</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C13" t="n">
+        <v>0.593684210526316</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.699492385786802</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.637206764866339</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" t="s">
         <v>29</v>
       </c>
       <c r="B14" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="1">
-        <v>1.6843971631205701</v>
-      </c>
-      <c r="D14" s="1">
-        <v>1.43251088534107</v>
-      </c>
-      <c r="E14" s="1">
-        <v>1.5693493150684901</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C14" t="n">
+        <v>1.68439716312057</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.42960812772134</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.56934931506849</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" t="s">
         <v>31</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="1">
-        <v>2.0780141843971598</v>
-      </c>
-      <c r="D15" s="1">
-        <v>1.96806966618287</v>
-      </c>
-      <c r="E15" s="1">
-        <v>2.0359589041095898</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C15" t="n">
+        <v>2.07801418439716</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1.96371552975327</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.03595890410959</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" t="s">
         <v>33</v>
       </c>
       <c r="B16" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" t="n">
         <v>2.6</v>
       </c>
-      <c r="D16" s="1">
-        <v>2.5805687203791501</v>
-      </c>
-      <c r="E16" s="1">
-        <v>2.5960526315789498</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D16" t="n">
+        <v>2.58056872037915</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2.59605263157895</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" t="s">
         <v>35</v>
       </c>
       <c r="B17" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="1">
-        <v>2.4911347517730502</v>
-      </c>
-      <c r="D17" s="1">
-        <v>3.5732946298983999</v>
-      </c>
-      <c r="E17" s="1">
-        <v>2.8501712328767099</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C17" t="n">
+        <v>2.49113475177305</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.5732946298984</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.85017123287671</v>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" t="s">
         <v>37</v>
       </c>
       <c r="B18" t="s">
         <v>38</v>
       </c>
-      <c r="C18">
+      <c r="C18" t="n">
         <v>15</v>
       </c>
-      <c r="D18">
+      <c r="D18" t="n">
         <v>19</v>
       </c>
-      <c r="E18">
+      <c r="E18" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19">
       <c r="A19" t="s">
         <v>39</v>
       </c>
       <c r="B19" t="s">
         <v>40</v>
       </c>
-      <c r="C19">
+      <c r="C19" t="n">
         <v>675</v>
       </c>
-      <c r="D19">
+      <c r="D19" t="n">
         <v>671</v>
       </c>
-      <c r="E19">
+      <c r="E19" t="n">
         <v>924</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20">
       <c r="A20" t="s">
         <v>41</v>
       </c>
       <c r="B20" t="s">
         <v>42</v>
       </c>
-      <c r="C20">
+      <c r="C20" t="n">
         <v>122</v>
       </c>
-      <c r="D20">
+      <c r="D20" t="n">
         <v>108</v>
       </c>
-      <c r="E20">
+      <c r="E20" t="n">
         <v>228</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>